<commit_message>
Resolve SRT vs. semiotics tension: Aprea grounds representación in Verón
Investigator confirmed Aprea (2006, Cap.3) founds the representation
concept in Verón's "La semiosis social" (Gedisa, 1987), not Moscovici/
Jodelet -- added to Bibliography_base.bib with the reasoning for why SRT
still fits this thesis's single-corpus (interview-only) design better than
Verón's multi-discourse apparatus, which Aprea needed because his corpus
crossed press + policy + teacher discourse. Logged in the research journal
and in fichas_lectura_representaciones_sociales.xlsx.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_representaciones_sociales.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_representaciones_sociales.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -519,6 +519,13 @@
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Actualización 2026-10-03: se agregaron 2 candidatos de Castorina (sugerido en el Ateneo para 'representaciones docente'), ambos sin leer y marcados PENDIENTE DE CONFIRMAR — verificá con tu directora/comité cuál de los dos es el texto que te recomendaron antes de leer, porque son dos líneas distintas de su obra (empírica sobre docentes de primaria vs. teórico-epistemológica general).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Actualización 2026-10-04: se resolvió la duda sobre si la psicología social era pertinente dado que (a) tu corpus es solo discurso de entrevistas y (b) Cabello/Aprea se paran desde la semiótica (Verón). Conclusión: (a) no es problema -- la TRS se estudia vía discurso igual que tu diseño; (b) Aprea usa Verón porque su corpus cruza 3 discursos (prensa, política pública, docentes) -- vos tenés un solo discurso, por eso la TRS se ajusta mejor a tu diseño. Ver fila de Verón (1987) más abajo -- es una aclaración de linaje teórico para Antecedentes, no una ficha de lectura pendiente.</t>
         </is>
       </c>
     </row>
@@ -536,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -803,6 +810,38 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="160" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Verón (1987), "La semiosis social: fragmentos de una teoría de la discursividad", Gedisa — NO es tu marco, es el de Aprea (aclaración, no lectura pendiente)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CONFIRMADO por vos (2026-10-04): Aprea funda la noción de representación en este texto de Verón, no en Moscovici/Jodelet. El aparato veroniano analiza discursividad social a través de condiciones de producción/reconocimiento, cruzando varios discursos a la vez (en el caso de Aprea: prensa, política pública, docentes). No necesitás leerlo para tu Marco Teórico — es para nombrar la diferencia de linaje en Antecedentes, no para adoptarlo.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>No hay cita textual necesaria — se cita el libro como referencia de la base teórica de Aprea, no como fuente de un concepto que vos vayas a usar.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Explica por qué Aprea necesitaba otro aparato: su corpus cruzaba 3 discursos (prensa + política pública + docentes) — exactamente lo que la sociosemiótica de Verón requiere para funcionar. Tu corpus es un solo discurso (docentes entrevistadas), sin ese cruce — por eso la TRS (que estudia cómo UN grupo representa UN objeto a través de SU propio discurso) se ajusta mejor a tu diseño que el aparato de Verón.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>El aparato analítico completo de Verón (condiciones de producción/reconocimiento, interdiscursividad) — no lo vas a aplicar, solo nombrar la diferencia de linaje teórico.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>No aplica (aclaración teórica, no ficha de lectura)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Register Aprea (2006) substantive findings, not just theoretical framing
Investigator shared the findings sections of Aprea's chapter (how teachers
represented TIC in 2001-2003: exteriority, quantitative-not-qualitative
change, collection/product split, the unanimously-rejected teacher-
substitution hypothesis). Added to antecedentes.md §1 with three concrete
parallels to this thesis's own codebook (imaginario_rol_docente_futuro,
ejemplo_centrado_producto_proceso/aprendizaje_explicitado_en_ejemplo,
limita_integracion_sustantiva) -- a cross-tech-generation continuity worth
flagging for the Discusión chapter. Also updated the matching ficha row
and added a short pointer in the Aprea2006 bib note.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_representaciones_sociales.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/fichas_lectura_representaciones_sociales.xlsx
@@ -682,7 +682,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="150" customHeight="1">
+    <row r="5" ht="260" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Aprea (2006), "Las representaciones de las TIC en relación con los procesos educativos", Cap. 3 en Cabello (coord.), "Yo con la computadora no tengo nada que ver", UNGS</t>
@@ -700,7 +700,8 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Es tu antecedente empírico más directo — mismo campo (docentes, CABA/conurbano, representaciones sobre tecnología educativa). Útil para el estado del arte (Cap. 1) y para argumentar por qué las entrevistas alcanzan para estudiar representaciones (ver tu pregunta sobre si faltan observaciones — Aprea trabaja con entrevistas + encuesta, no con observación de aula).</t>
+          <t>Es tu antecedente empírico más directo — mismo campo (docentes, CABA/conurbano, representaciones sobre tecnología educativa). Útil para el estado del arte (Cap. 1) y para argumentar por qué las entrevistas alcanzan para estudiar representaciones (ver tu pregunta sobre si faltan observaciones — Aprea trabaja con entrevistas + encuesta, no con observación de aula).
+ACTUALIZADO 2026-10-13 (hallazgos, no solo marco teórico, compartidos por la investigadora): Aprea rechaza por unanimidad, en su corpus, la hipótesis de sustitución del docente por el dispositivo -- los maestros se reservan el rol de "guías"/"orientadores". Esto es casi literal al código `imaginario_rol_docente_futuro` de esta tesis (ejemplo ya en el codebook: "El docente va a tener que ser más un guía que alguien que transmite contenido") -- continuidad de la misma representación a 20 años y dos tecnologías distintas, dato fuerte para la Discusión. También conecta: la separación recolección-de-información/generación-de-producto sin continuidad (Aprea) con `ejemplo_centrado_producto_proceso` y `aprendizaje_explicitado_en_ejemplo` (0/15 en este corpus); y el "achatamiento" de la información como cantidad, no transformación cualitativa, con `limita_integracion_sustantiva` (Dimensión 4). Detalle completo en `antecedentes.md` §1.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">

</xml_diff>